<commit_message>
Add pattern-based likely emails for franchises without a published email
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3ukMUJQ3Jbp8uBVM3LeTR
</commit_message>
<xml_diff>
--- a/Fish_Window_Cleaning_Locations.xlsx
+++ b/Fish_Window_Cleaning_Locations.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Locations'!$A$1:$K$262</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Locations'!$A$1:$M$262</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K262"/>
+  <dimension ref="A1:M262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,9 @@
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -518,10 +520,20 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>Email(s)</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
+          <t>Email(s) - Published</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Likely Email (pattern, unverified)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Alternate Guess (co-owner)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Location Page URL</t>
         </is>
@@ -574,7 +586,13 @@
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>tharper@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr"/>
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Alabaster-AL-3199/</t>
         </is>
@@ -627,7 +645,17 @@
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>hzein@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>ysharfi@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Huntsville-AL-335/</t>
         </is>
@@ -680,7 +708,13 @@
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>dmiller@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr"/>
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Jonesboro-AR-3250/</t>
         </is>
@@ -733,7 +767,13 @@
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>jholmstrom@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr"/>
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Fayetteville-AR-3137/</t>
         </is>
@@ -786,7 +826,13 @@
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>esmith@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr"/>
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Phoenix-AZ-3006/</t>
         </is>
@@ -839,7 +885,13 @@
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>jguidi@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Tempe-AZ-3279/</t>
         </is>
@@ -892,7 +944,17 @@
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>cgallegos@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>jgallegos@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Chandler-AZ-3276/</t>
         </is>
@@ -945,7 +1007,13 @@
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>jislas@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr"/>
+      <c r="M9" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Tucson-AZ-880/</t>
         </is>
@@ -998,7 +1066,13 @@
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr"/>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>htse@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Concord-CA-3051/</t>
         </is>
@@ -1051,7 +1125,13 @@
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>atse@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr"/>
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Fremont-CA-3291/</t>
         </is>
@@ -1104,7 +1184,13 @@
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr"/>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>kjones@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr"/>
+      <c r="M12" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Fontana-CA-3080/</t>
         </is>
@@ -1157,7 +1243,13 @@
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>jrieman@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr"/>
+      <c r="M13" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Rocklin-CA-3292/</t>
         </is>
@@ -1210,7 +1302,13 @@
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr"/>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>kjones@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr"/>
+      <c r="M14" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Redlands-CA-618/</t>
         </is>
@@ -1263,7 +1361,13 @@
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr"/>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>jmay@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr"/>
+      <c r="M15" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Laguna-Hills-CA-3035/</t>
         </is>
@@ -1316,7 +1420,13 @@
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>apartida@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr"/>
+      <c r="M16" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Downey-CA-3236/</t>
         </is>
@@ -1369,7 +1479,13 @@
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr"/>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>tchesney@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr"/>
+      <c r="M17" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Los-Angeles-CA-611/</t>
         </is>
@@ -1422,7 +1538,13 @@
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>kmay@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr"/>
+      <c r="M18" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Irvine-CA-3086/</t>
         </is>
@@ -1475,7 +1597,13 @@
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr"/>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>mduong@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr"/>
+      <c r="M19" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Arcadia-CA-3268/</t>
         </is>
@@ -1528,7 +1656,17 @@
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr"/>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>kjones@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>mjones@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Rancho-Cucamonga-CA-3231/</t>
         </is>
@@ -1581,7 +1719,13 @@
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr"/>
-      <c r="K21" s="3" t="inlineStr">
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>etamodaran@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr"/>
+      <c r="M21" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Sacramento-CA-889/</t>
         </is>
@@ -1634,7 +1778,13 @@
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr"/>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>amiller@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr"/>
+      <c r="M22" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Oceanside-CA-3173/</t>
         </is>
@@ -1687,7 +1837,17 @@
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr"/>
-      <c r="K23" s="3" t="inlineStr">
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>pthomas@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>rthomas@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/San-Diego-CA-3177/</t>
         </is>
@@ -1740,7 +1900,13 @@
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr"/>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>jnealon@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr"/>
+      <c r="M24" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Woodland-Hills-CA-3114/</t>
         </is>
@@ -1793,7 +1959,13 @@
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr"/>
-      <c r="K25" s="3" t="inlineStr">
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>bgawick@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr"/>
+      <c r="M25" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/San-Rafael-CA-3088/</t>
         </is>
@@ -1846,7 +2018,13 @@
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr"/>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>jrubin@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr"/>
+      <c r="M26" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Santa-Barbara-CA-3037/</t>
         </is>
@@ -1899,7 +2077,13 @@
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr"/>
-      <c r="K27" s="3" t="inlineStr">
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>cpolk@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr"/>
+      <c r="M27" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Santa-Clara-CA-3230/</t>
         </is>
@@ -1952,7 +2136,13 @@
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr"/>
-      <c r="K28" s="3" t="inlineStr">
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>bgawick@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr"/>
+      <c r="M28" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Santa-Rosa-CA-3107/</t>
         </is>
@@ -2005,7 +2195,13 @@
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr"/>
-      <c r="K29" s="3" t="inlineStr">
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>rtriffo@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr"/>
+      <c r="M29" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Murrieta-CA-887/</t>
         </is>
@@ -2058,7 +2254,17 @@
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr"/>
-      <c r="K30" s="3" t="inlineStr">
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>scuster@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>gcuster@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Lancaster-CA-805/</t>
         </is>
@@ -2111,7 +2317,13 @@
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr"/>
-      <c r="K31" s="3" t="inlineStr">
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>spropp@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr"/>
+      <c r="M31" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Westminster-CO-3270/</t>
         </is>
@@ -2164,7 +2376,13 @@
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr"/>
-      <c r="K32" s="3" t="inlineStr">
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>jrowsell@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr"/>
+      <c r="M32" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Denver-CO-2080/</t>
         </is>
@@ -2217,7 +2435,13 @@
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr"/>
-      <c r="K33" s="3" t="inlineStr">
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>mphillips@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr"/>
+      <c r="M33" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Colorado-Springs-CO-832/</t>
         </is>
@@ -2270,7 +2494,13 @@
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr"/>
-      <c r="K34" s="3" t="inlineStr">
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>ecornett@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr"/>
+      <c r="M34" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Denver-CO-735/</t>
         </is>
@@ -2323,7 +2553,13 @@
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr"/>
-      <c r="K35" s="3" t="inlineStr">
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>lminter@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr"/>
+      <c r="M35" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Fort-Collins-CO-850/</t>
         </is>
@@ -2376,7 +2612,13 @@
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr"/>
-      <c r="K36" s="3" t="inlineStr">
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>pwise@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr"/>
+      <c r="M36" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Littleton-CO-623/</t>
         </is>
@@ -2421,7 +2663,13 @@
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr"/>
-      <c r="K37" s="3" t="inlineStr">
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>mphillips@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr"/>
+      <c r="M37" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Pueblo-CO-882/</t>
         </is>
@@ -2474,7 +2722,13 @@
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr"/>
-      <c r="K38" s="3" t="inlineStr">
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>bmendes@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr"/>
+      <c r="M38" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Manchester-CT-631/</t>
         </is>
@@ -2527,7 +2781,13 @@
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr"/>
-      <c r="K39" s="3" t="inlineStr">
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>korourke@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr"/>
+      <c r="M39" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/New-Haven-CT-871/</t>
         </is>
@@ -2580,7 +2840,13 @@
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr"/>
-      <c r="K40" s="3" t="inlineStr">
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>jracicot@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr"/>
+      <c r="M40" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Southeast-CT-3151/</t>
         </is>
@@ -2633,7 +2899,13 @@
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr"/>
-      <c r="K41" s="3" t="inlineStr">
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>hkhan@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr"/>
+      <c r="M41" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Dover-DE-677/</t>
         </is>
@@ -2686,7 +2958,17 @@
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr"/>
-      <c r="K42" s="3" t="inlineStr">
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>mhannum@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>dhannum@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Wilmington-DE-3215/</t>
         </is>
@@ -2743,7 +3025,9 @@
           <t>mhaberman@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K43" s="3" t="inlineStr">
+      <c r="K43" s="4" t="inlineStr"/>
+      <c r="L43" s="4" t="inlineStr"/>
+      <c r="M43" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Boca-Raton-655/</t>
         </is>
@@ -2796,7 +3080,13 @@
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr"/>
-      <c r="K44" s="3" t="inlineStr">
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>mcarter@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr"/>
+      <c r="M44" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Bradenton-FL-3049/</t>
         </is>
@@ -2845,7 +3135,9 @@
           <t>atorres@fishwindowcleaning.com; gbiltis@fishwindowcleaning.com; jennacompton@fishwindowcleaning.com; joeycompton@fishwindowcleaning.com; mhaberman@fishwindowcleaning.com; mvillanueva@fishwindowcleaning.com; ykhan@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K45" s="3" t="inlineStr">
+      <c r="K45" s="4" t="inlineStr"/>
+      <c r="L45" s="4" t="inlineStr"/>
+      <c r="M45" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/sefl/</t>
         </is>
@@ -2898,7 +3190,13 @@
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr"/>
-      <c r="K46" s="3" t="inlineStr">
+      <c r="K46" s="4" t="inlineStr">
+        <is>
+          <t>dgalloway@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L46" s="4" t="inlineStr"/>
+      <c r="M46" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Clearwater-FL-3096/</t>
         </is>
@@ -2955,7 +3253,9 @@
           <t>gbiltis@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K47" s="3" t="inlineStr">
+      <c r="K47" s="4" t="inlineStr"/>
+      <c r="L47" s="4" t="inlineStr"/>
+      <c r="M47" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Pompano-Beach-FL-3079/</t>
         </is>
@@ -3012,7 +3312,9 @@
           <t>ykhan@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K48" s="3" t="inlineStr">
+      <c r="K48" s="4" t="inlineStr"/>
+      <c r="L48" s="4" t="inlineStr"/>
+      <c r="M48" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Coral-Gables-FL-3147/</t>
         </is>
@@ -3069,7 +3371,9 @@
           <t>rboals@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K49" s="3" t="inlineStr">
+      <c r="K49" s="4" t="inlineStr"/>
+      <c r="L49" s="4" t="inlineStr"/>
+      <c r="M49" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Daytona-Beach-FL-876/</t>
         </is>
@@ -3122,7 +3426,13 @@
         </is>
       </c>
       <c r="J50" s="4" t="inlineStr"/>
-      <c r="K50" s="3" t="inlineStr">
+      <c r="K50" s="4" t="inlineStr">
+        <is>
+          <t>dlafaire@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L50" s="4" t="inlineStr"/>
+      <c r="M50" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Destin-FL-3249/</t>
         </is>
@@ -3179,7 +3489,9 @@
           <t>jennacompton@fishwindowcleaning.com; joeycompton@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K51" s="3" t="inlineStr">
+      <c r="K51" s="4" t="inlineStr"/>
+      <c r="L51" s="4" t="inlineStr"/>
+      <c r="M51" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Fort-Lauderdale-FL-311/</t>
         </is>
@@ -3232,7 +3544,13 @@
         </is>
       </c>
       <c r="J52" s="4" t="inlineStr"/>
-      <c r="K52" s="3" t="inlineStr">
+      <c r="K52" s="4" t="inlineStr">
+        <is>
+          <t>dweissinger@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L52" s="4" t="inlineStr"/>
+      <c r="M52" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Fort-Myers-Cape-Coral-FL-3163/</t>
         </is>
@@ -3285,7 +3603,13 @@
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr"/>
-      <c r="K53" s="3" t="inlineStr">
+      <c r="K53" s="4" t="inlineStr">
+        <is>
+          <t>crobinson@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L53" s="4" t="inlineStr"/>
+      <c r="M53" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Tampa-FL-3187/</t>
         </is>
@@ -3338,7 +3662,13 @@
         </is>
       </c>
       <c r="J54" s="4" t="inlineStr"/>
-      <c r="K54" s="3" t="inlineStr">
+      <c r="K54" s="4" t="inlineStr">
+        <is>
+          <t>crobinson@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L54" s="4" t="inlineStr"/>
+      <c r="M54" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Tampa-FL-3253/</t>
         </is>
@@ -3391,7 +3721,17 @@
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr"/>
-      <c r="K55" s="3" t="inlineStr">
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>dfrazier@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>cfrazier@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M55" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Port-Saint-Lucie-FL-3181/</t>
         </is>
@@ -3448,7 +3788,9 @@
           <t>rzanelly@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K56" s="3" t="inlineStr">
+      <c r="K56" s="4" t="inlineStr"/>
+      <c r="L56" s="4" t="inlineStr"/>
+      <c r="M56" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Kissimmee-FL-3159/</t>
         </is>
@@ -3501,7 +3843,17 @@
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr"/>
-      <c r="K57" s="3" t="inlineStr">
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>jzeigler@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>mzeigler@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M57" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Lakeland-FL-3272/</t>
         </is>
@@ -3554,7 +3906,13 @@
         </is>
       </c>
       <c r="J58" s="4" t="inlineStr"/>
-      <c r="K58" s="3" t="inlineStr">
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>ikennedy@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L58" s="4" t="inlineStr"/>
+      <c r="M58" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Melbourne-FL-852/</t>
         </is>
@@ -3611,7 +3969,9 @@
           <t>atorres@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K59" s="3" t="inlineStr">
+      <c r="K59" s="4" t="inlineStr"/>
+      <c r="L59" s="4" t="inlineStr"/>
+      <c r="M59" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Miami-FL-3016/</t>
         </is>
@@ -3668,7 +4028,9 @@
           <t>mvillanueva@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K60" s="3" t="inlineStr">
+      <c r="K60" s="4" t="inlineStr"/>
+      <c r="L60" s="4" t="inlineStr"/>
+      <c r="M60" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Miami-FL-3164/</t>
         </is>
@@ -3721,7 +4083,13 @@
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr"/>
-      <c r="K61" s="3" t="inlineStr">
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>dweissinger@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L61" s="4" t="inlineStr"/>
+      <c r="M61" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Naples-FL-3260/</t>
         </is>
@@ -3774,7 +4142,13 @@
         </is>
       </c>
       <c r="J62" s="4" t="inlineStr"/>
-      <c r="K62" s="3" t="inlineStr">
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>sjantz@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L62" s="4" t="inlineStr"/>
+      <c r="M62" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Jacksonville-FL-105/</t>
         </is>
@@ -3827,7 +4201,13 @@
         </is>
       </c>
       <c r="J63" s="4" t="inlineStr"/>
-      <c r="K63" s="3" t="inlineStr">
+      <c r="K63" s="4" t="inlineStr">
+        <is>
+          <t>rzanelly@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L63" s="4" t="inlineStr"/>
+      <c r="M63" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Orlando-FL-3259/</t>
         </is>
@@ -3884,7 +4264,9 @@
           <t>rboals@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K64" s="3" t="inlineStr">
+      <c r="K64" s="4" t="inlineStr"/>
+      <c r="L64" s="4" t="inlineStr"/>
+      <c r="M64" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Orlando-FL-360/</t>
         </is>
@@ -3937,7 +4319,17 @@
         </is>
       </c>
       <c r="J65" s="4" t="inlineStr"/>
-      <c r="K65" s="3" t="inlineStr">
+      <c r="K65" s="4" t="inlineStr">
+        <is>
+          <t>ctalbert@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L65" s="4" t="inlineStr">
+        <is>
+          <t>jtalbert@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M65" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Saint-Petersburg-FL-3263/</t>
         </is>
@@ -3990,7 +4382,13 @@
         </is>
       </c>
       <c r="J66" s="4" t="inlineStr"/>
-      <c r="K66" s="3" t="inlineStr">
+      <c r="K66" s="4" t="inlineStr">
+        <is>
+          <t>mcombs@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L66" s="4" t="inlineStr"/>
+      <c r="M66" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Sarasota-FL-3129/</t>
         </is>
@@ -4043,7 +4441,9 @@
           <t>mdambrosio@fishwindowcleaning.com; rboals@fishwindowcleaning.com; rzanelly@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K67" s="3" t="inlineStr">
+      <c r="K67" s="4" t="inlineStr"/>
+      <c r="L67" s="4" t="inlineStr"/>
+      <c r="M67" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/cfl/</t>
         </is>
@@ -4096,7 +4496,13 @@
         </is>
       </c>
       <c r="J68" s="4" t="inlineStr"/>
-      <c r="K68" s="3" t="inlineStr">
+      <c r="K68" s="4" t="inlineStr">
+        <is>
+          <t>mpreston@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L68" s="4" t="inlineStr"/>
+      <c r="M68" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Tallahassee-FL-3039/</t>
         </is>
@@ -4149,7 +4555,13 @@
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr"/>
-      <c r="K69" s="3" t="inlineStr">
+      <c r="K69" s="4" t="inlineStr">
+        <is>
+          <t>klowe@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L69" s="4" t="inlineStr"/>
+      <c r="M69" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Wesley-Chapel-FL-3225/</t>
         </is>
@@ -4206,7 +4618,9 @@
           <t>mdambrosio@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K70" s="3" t="inlineStr">
+      <c r="K70" s="4" t="inlineStr"/>
+      <c r="L70" s="4" t="inlineStr"/>
+      <c r="M70" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Orlando-FL-3152/</t>
         </is>
@@ -4263,7 +4677,9 @@
           <t>lsimons@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K71" s="3" t="inlineStr">
+      <c r="K71" s="4" t="inlineStr"/>
+      <c r="L71" s="4" t="inlineStr"/>
+      <c r="M71" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Marietta-GA-854/</t>
         </is>
@@ -4320,7 +4736,9 @@
           <t>jparham@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K72" s="3" t="inlineStr">
+      <c r="K72" s="4" t="inlineStr"/>
+      <c r="L72" s="4" t="inlineStr"/>
+      <c r="M72" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Athens-GA-3246/</t>
         </is>
@@ -4369,7 +4787,9 @@
           <t>bwanderson@fishwindowcleaning.com; gjordan@fishwindowcleaning.com; jparham@fishwindowcleaning.com; jworsham@fishwindowcleaning.com; lsimons@fishwindowcleaning.com; mquadri@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K73" s="3" t="inlineStr">
+      <c r="K73" s="4" t="inlineStr"/>
+      <c r="L73" s="4" t="inlineStr"/>
+      <c r="M73" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Atlanta/</t>
         </is>
@@ -4426,7 +4846,9 @@
           <t>gjordan@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K74" s="3" t="inlineStr">
+      <c r="K74" s="4" t="inlineStr"/>
+      <c r="L74" s="4" t="inlineStr"/>
+      <c r="M74" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Atlanta-GA-643/</t>
         </is>
@@ -4479,7 +4901,17 @@
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr"/>
-      <c r="K75" s="3" t="inlineStr">
+      <c r="K75" s="4" t="inlineStr">
+        <is>
+          <t>aryan@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L75" s="4" t="inlineStr">
+        <is>
+          <t>jryan@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M75" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Augusta-GA-3022/</t>
         </is>
@@ -4532,7 +4964,13 @@
         </is>
       </c>
       <c r="J76" s="4" t="inlineStr"/>
-      <c r="K76" s="3" t="inlineStr">
+      <c r="K76" s="4" t="inlineStr">
+        <is>
+          <t>nhill@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L76" s="4" t="inlineStr"/>
+      <c r="M76" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Columbus-GA-3209/</t>
         </is>
@@ -4589,7 +5027,9 @@
           <t>mquadri@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K77" s="3" t="inlineStr">
+      <c r="K77" s="4" t="inlineStr"/>
+      <c r="L77" s="4" t="inlineStr"/>
+      <c r="M77" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Atlanta-GA-3224/</t>
         </is>
@@ -4646,7 +5086,9 @@
           <t>jworsham@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K78" s="3" t="inlineStr">
+      <c r="K78" s="4" t="inlineStr"/>
+      <c r="L78" s="4" t="inlineStr"/>
+      <c r="M78" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Gainesville-GA-3058/</t>
         </is>
@@ -4703,7 +5145,9 @@
           <t>jparham@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K79" s="3" t="inlineStr">
+      <c r="K79" s="4" t="inlineStr"/>
+      <c r="L79" s="4" t="inlineStr"/>
+      <c r="M79" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Lake-Oconee-GA-3246/</t>
         </is>
@@ -4756,7 +5200,17 @@
         </is>
       </c>
       <c r="J80" s="4" t="inlineStr"/>
-      <c r="K80" s="3" t="inlineStr">
+      <c r="K80" s="4" t="inlineStr">
+        <is>
+          <t>rrowe@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L80" s="4" t="inlineStr">
+        <is>
+          <t>ibratianu@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M80" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Hilton-Head-SC-30170/</t>
         </is>
@@ -4809,7 +5263,13 @@
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr"/>
-      <c r="K81" s="3" t="inlineStr">
+      <c r="K81" s="4" t="inlineStr">
+        <is>
+          <t>jparham@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L81" s="4" t="inlineStr"/>
+      <c r="M81" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Loganville-GA-3018/</t>
         </is>
@@ -4866,7 +5326,9 @@
           <t>bwanderson@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K82" s="3" t="inlineStr">
+      <c r="K82" s="4" t="inlineStr"/>
+      <c r="L82" s="4" t="inlineStr"/>
+      <c r="M82" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/McDonough-GA-3218/</t>
         </is>
@@ -4919,7 +5381,17 @@
         </is>
       </c>
       <c r="J83" s="4" t="inlineStr"/>
-      <c r="K83" s="3" t="inlineStr">
+      <c r="K83" s="4" t="inlineStr">
+        <is>
+          <t>rrowe@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L83" s="4" t="inlineStr">
+        <is>
+          <t>ibratianu@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M83" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Savannah-GA-3017/</t>
         </is>
@@ -4972,7 +5444,17 @@
         </is>
       </c>
       <c r="J84" s="4" t="inlineStr"/>
-      <c r="K84" s="3" t="inlineStr">
+      <c r="K84" s="4" t="inlineStr">
+        <is>
+          <t>cmccallum@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L84" s="4" t="inlineStr">
+        <is>
+          <t>lmccallum@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M84" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Cedar-Falls-IA-3143/</t>
         </is>
@@ -5025,7 +5507,13 @@
         </is>
       </c>
       <c r="J85" s="4" t="inlineStr"/>
-      <c r="K85" s="3" t="inlineStr">
+      <c r="K85" s="4" t="inlineStr">
+        <is>
+          <t>ealatorre@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L85" s="4" t="inlineStr"/>
+      <c r="M85" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Cedar-Rapids-IA-3204/</t>
         </is>
@@ -5078,7 +5566,13 @@
         </is>
       </c>
       <c r="J86" s="4" t="inlineStr"/>
-      <c r="K86" s="3" t="inlineStr">
+      <c r="K86" s="4" t="inlineStr">
+        <is>
+          <t>twhite@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L86" s="4" t="inlineStr"/>
+      <c r="M86" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Des-Moines-IA-3061/</t>
         </is>
@@ -5135,7 +5629,9 @@
           <t>dweishar@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K87" s="3" t="inlineStr">
+      <c r="K87" s="4" t="inlineStr"/>
+      <c r="L87" s="4" t="inlineStr"/>
+      <c r="M87" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Chicago-Western-Southern-Suburbs-3277/</t>
         </is>
@@ -5184,7 +5680,9 @@
           <t>admin2715@fishwindowcleaning.com; cstraka@fishwindowcleaning.com; djaggers@fishwindowcleaning.com; dweishar@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K88" s="3" t="inlineStr">
+      <c r="K88" s="4" t="inlineStr"/>
+      <c r="L88" s="4" t="inlineStr"/>
+      <c r="M88" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Chicago/</t>
         </is>
@@ -5241,7 +5739,9 @@
           <t>djaggers@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K89" s="3" t="inlineStr">
+      <c r="K89" s="4" t="inlineStr"/>
+      <c r="L89" s="4" t="inlineStr"/>
+      <c r="M89" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Chicagoland-IL-3289/</t>
         </is>
@@ -5294,7 +5794,13 @@
         </is>
       </c>
       <c r="J90" s="4" t="inlineStr"/>
-      <c r="K90" s="3" t="inlineStr">
+      <c r="K90" s="4" t="inlineStr">
+        <is>
+          <t>cstraka@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L90" s="4" t="inlineStr"/>
+      <c r="M90" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Waukegan-IL-30630/</t>
         </is>
@@ -5351,7 +5857,9 @@
           <t>admin2715@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K91" s="3" t="inlineStr">
+      <c r="K91" s="4" t="inlineStr"/>
+      <c r="L91" s="4" t="inlineStr"/>
+      <c r="M91" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Chicago-IL-715/</t>
         </is>
@@ -5404,7 +5912,13 @@
         </is>
       </c>
       <c r="J92" s="4" t="inlineStr"/>
-      <c r="K92" s="3" t="inlineStr">
+      <c r="K92" s="4" t="inlineStr">
+        <is>
+          <t>jkesler@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L92" s="4" t="inlineStr"/>
+      <c r="M92" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Metro-East-IL-3287/</t>
         </is>
@@ -5457,7 +5971,13 @@
         </is>
       </c>
       <c r="J93" s="4" t="inlineStr"/>
-      <c r="K93" s="3" t="inlineStr">
+      <c r="K93" s="4" t="inlineStr">
+        <is>
+          <t>wwright@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L93" s="4" t="inlineStr"/>
+      <c r="M93" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Joliet-IL-3247/</t>
         </is>
@@ -5510,7 +6030,13 @@
         </is>
       </c>
       <c r="J94" s="4" t="inlineStr"/>
-      <c r="K94" s="3" t="inlineStr">
+      <c r="K94" s="4" t="inlineStr">
+        <is>
+          <t>blanghans@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L94" s="4" t="inlineStr"/>
+      <c r="M94" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Oswego-IL-3285/</t>
         </is>
@@ -5563,7 +6089,13 @@
         </is>
       </c>
       <c r="J95" s="4" t="inlineStr"/>
-      <c r="K95" s="3" t="inlineStr">
+      <c r="K95" s="4" t="inlineStr">
+        <is>
+          <t>wmoses@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L95" s="4" t="inlineStr"/>
+      <c r="M95" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Peoria-IL-879/</t>
         </is>
@@ -5616,7 +6148,17 @@
         </is>
       </c>
       <c r="J96" s="4" t="inlineStr"/>
-      <c r="K96" s="3" t="inlineStr">
+      <c r="K96" s="4" t="inlineStr">
+        <is>
+          <t>jspude@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L96" s="4" t="inlineStr">
+        <is>
+          <t>dspude@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M96" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Rockford-IL-30640/</t>
         </is>
@@ -5669,7 +6211,13 @@
         </is>
       </c>
       <c r="J97" s="4" t="inlineStr"/>
-      <c r="K97" s="3" t="inlineStr">
+      <c r="K97" s="4" t="inlineStr">
+        <is>
+          <t>trichardson@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L97" s="4" t="inlineStr"/>
+      <c r="M97" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Bloomington-IN-3120/</t>
         </is>
@@ -5722,7 +6270,17 @@
         </is>
       </c>
       <c r="J98" s="4" t="inlineStr"/>
-      <c r="K98" s="3" t="inlineStr">
+      <c r="K98" s="4" t="inlineStr">
+        <is>
+          <t>mbaker@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L98" s="4" t="inlineStr">
+        <is>
+          <t>cbaker@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M98" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Indianapolis-IN-3161/</t>
         </is>
@@ -5775,7 +6333,17 @@
         </is>
       </c>
       <c r="J99" s="4" t="inlineStr"/>
-      <c r="K99" s="3" t="inlineStr">
+      <c r="K99" s="4" t="inlineStr">
+        <is>
+          <t>bsoots@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L99" s="4" t="inlineStr">
+        <is>
+          <t>jsoots@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M99" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Indianapolis-IN-858/</t>
         </is>
@@ -5828,7 +6396,17 @@
         </is>
       </c>
       <c r="J100" s="4" t="inlineStr"/>
-      <c r="K100" s="3" t="inlineStr">
+      <c r="K100" s="4" t="inlineStr">
+        <is>
+          <t>dmejan@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L100" s="4" t="inlineStr">
+        <is>
+          <t>cmejan@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M100" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Crown-Point-IN-3205/</t>
         </is>
@@ -5881,7 +6459,17 @@
         </is>
       </c>
       <c r="J101" s="4" t="inlineStr"/>
-      <c r="K101" s="3" t="inlineStr">
+      <c r="K101" s="4" t="inlineStr">
+        <is>
+          <t>kbrown@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L101" s="4" t="inlineStr">
+        <is>
+          <t>nbrown@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M101" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/South-Bend-IN-3124/</t>
         </is>
@@ -5934,7 +6522,17 @@
         </is>
       </c>
       <c r="J102" s="4" t="inlineStr"/>
-      <c r="K102" s="3" t="inlineStr">
+      <c r="K102" s="4" t="inlineStr">
+        <is>
+          <t>jcoons@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L102" s="4" t="inlineStr">
+        <is>
+          <t>acoons@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M102" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Terre-Haute-IN-3245/</t>
         </is>
@@ -5987,7 +6585,13 @@
         </is>
       </c>
       <c r="J103" s="4" t="inlineStr"/>
-      <c r="K103" s="3" t="inlineStr">
+      <c r="K103" s="4" t="inlineStr">
+        <is>
+          <t>bkuhn@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L103" s="4" t="inlineStr"/>
+      <c r="M103" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Indianapolis-IN-3084/</t>
         </is>
@@ -6040,7 +6644,13 @@
         </is>
       </c>
       <c r="J104" s="4" t="inlineStr"/>
-      <c r="K104" s="3" t="inlineStr">
+      <c r="K104" s="4" t="inlineStr">
+        <is>
+          <t>sroach@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L104" s="4" t="inlineStr"/>
+      <c r="M104" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/628/</t>
         </is>
@@ -6093,7 +6703,17 @@
         </is>
       </c>
       <c r="J105" s="4" t="inlineStr"/>
-      <c r="K105" s="3" t="inlineStr">
+      <c r="K105" s="4" t="inlineStr">
+        <is>
+          <t>mmckee@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L105" s="4" t="inlineStr">
+        <is>
+          <t>dmckee@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M105" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Wichita-KS-888/</t>
         </is>
@@ -6146,7 +6766,13 @@
         </is>
       </c>
       <c r="J106" s="4" t="inlineStr"/>
-      <c r="K106" s="3" t="inlineStr">
+      <c r="K106" s="4" t="inlineStr">
+        <is>
+          <t>mdebord@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L106" s="4" t="inlineStr"/>
+      <c r="M106" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Lexington-KY-181/</t>
         </is>
@@ -6199,7 +6825,17 @@
         </is>
       </c>
       <c r="J107" s="4" t="inlineStr"/>
-      <c r="K107" s="3" t="inlineStr">
+      <c r="K107" s="4" t="inlineStr">
+        <is>
+          <t>bwathen@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L107" s="4" t="inlineStr">
+        <is>
+          <t>dbaker@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M107" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Louisville-KY-685/</t>
         </is>
@@ -6252,7 +6888,17 @@
         </is>
       </c>
       <c r="J108" s="4" t="inlineStr"/>
-      <c r="K108" s="3" t="inlineStr">
+      <c r="K108" s="4" t="inlineStr">
+        <is>
+          <t>jnegron@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L108" s="4" t="inlineStr">
+        <is>
+          <t>nnegron@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M108" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Shreveport-LA-3131/</t>
         </is>
@@ -6305,7 +6951,13 @@
         </is>
       </c>
       <c r="J109" s="4" t="inlineStr"/>
-      <c r="K109" s="3" t="inlineStr">
+      <c r="K109" s="4" t="inlineStr">
+        <is>
+          <t>broberts@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L109" s="4" t="inlineStr"/>
+      <c r="M109" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Hammond-LA-834/</t>
         </is>
@@ -6358,7 +7010,13 @@
         </is>
       </c>
       <c r="J110" s="4" t="inlineStr"/>
-      <c r="K110" s="3" t="inlineStr">
+      <c r="K110" s="4" t="inlineStr">
+        <is>
+          <t>cmatherne@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L110" s="4" t="inlineStr"/>
+      <c r="M110" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Lafayette-LA-3150/</t>
         </is>
@@ -6411,7 +7069,17 @@
         </is>
       </c>
       <c r="J111" s="4" t="inlineStr"/>
-      <c r="K111" s="3" t="inlineStr">
+      <c r="K111" s="4" t="inlineStr">
+        <is>
+          <t>lreinagel@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L111" s="4" t="inlineStr">
+        <is>
+          <t>jreinagel@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M111" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/New-Orleans-LA-3105/</t>
         </is>
@@ -6464,7 +7132,13 @@
         </is>
       </c>
       <c r="J112" s="4" t="inlineStr"/>
-      <c r="K112" s="3" t="inlineStr">
+      <c r="K112" s="4" t="inlineStr">
+        <is>
+          <t>bdower@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L112" s="4" t="inlineStr"/>
+      <c r="M112" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Amesbury-MA-3050/</t>
         </is>
@@ -6517,7 +7191,13 @@
         </is>
       </c>
       <c r="J113" s="4" t="inlineStr"/>
-      <c r="K113" s="3" t="inlineStr">
+      <c r="K113" s="4" t="inlineStr">
+        <is>
+          <t>pthurston@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L113" s="4" t="inlineStr"/>
+      <c r="M113" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Lawrence-MA-3850/</t>
         </is>
@@ -6562,7 +7242,13 @@
         </is>
       </c>
       <c r="J114" s="4" t="inlineStr"/>
-      <c r="K114" s="3" t="inlineStr">
+      <c r="K114" s="4" t="inlineStr">
+        <is>
+          <t>npierce@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L114" s="4" t="inlineStr"/>
+      <c r="M114" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Cambridge-MA-300/</t>
         </is>
@@ -6615,7 +7301,13 @@
         </is>
       </c>
       <c r="J115" s="4" t="inlineStr"/>
-      <c r="K115" s="3" t="inlineStr">
+      <c r="K115" s="4" t="inlineStr">
+        <is>
+          <t>agarrett@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L115" s="4" t="inlineStr"/>
+      <c r="M115" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Hopedale-MA-899/</t>
         </is>
@@ -6668,7 +7360,13 @@
         </is>
       </c>
       <c r="J116" s="4" t="inlineStr"/>
-      <c r="K116" s="3" t="inlineStr">
+      <c r="K116" s="4" t="inlineStr">
+        <is>
+          <t>npierce@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L116" s="4" t="inlineStr"/>
+      <c r="M116" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Boston-North-Shore-MA-595/</t>
         </is>
@@ -6721,7 +7419,13 @@
         </is>
       </c>
       <c r="J117" s="4" t="inlineStr"/>
-      <c r="K117" s="3" t="inlineStr">
+      <c r="K117" s="4" t="inlineStr">
+        <is>
+          <t>npierce@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L117" s="4" t="inlineStr"/>
+      <c r="M117" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Boston-South-Shore-MA-615/</t>
         </is>
@@ -6774,7 +7478,13 @@
         </is>
       </c>
       <c r="J118" s="4" t="inlineStr"/>
-      <c r="K118" s="3" t="inlineStr">
+      <c r="K118" s="4" t="inlineStr">
+        <is>
+          <t>dbackus@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L118" s="4" t="inlineStr"/>
+      <c r="M118" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Leominster-MA-410/</t>
         </is>
@@ -6827,7 +7537,13 @@
         </is>
       </c>
       <c r="J119" s="4" t="inlineStr"/>
-      <c r="K119" s="3" t="inlineStr">
+      <c r="K119" s="4" t="inlineStr">
+        <is>
+          <t>ddibiase@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L119" s="4" t="inlineStr"/>
+      <c r="M119" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Brockton-MA-3104/</t>
         </is>
@@ -6880,7 +7596,13 @@
         </is>
       </c>
       <c r="J120" s="4" t="inlineStr"/>
-      <c r="K120" s="3" t="inlineStr">
+      <c r="K120" s="4" t="inlineStr">
+        <is>
+          <t>mkhan@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L120" s="4" t="inlineStr"/>
+      <c r="M120" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Ellicott-City-MD-3004/</t>
         </is>
@@ -6933,7 +7655,13 @@
         </is>
       </c>
       <c r="J121" s="4" t="inlineStr"/>
-      <c r="K121" s="3" t="inlineStr">
+      <c r="K121" s="4" t="inlineStr">
+        <is>
+          <t>smerther@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L121" s="4" t="inlineStr"/>
+      <c r="M121" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Laurel-MD-696/</t>
         </is>
@@ -6986,7 +7714,13 @@
         </is>
       </c>
       <c r="J122" s="4" t="inlineStr"/>
-      <c r="K122" s="3" t="inlineStr">
+      <c r="K122" s="4" t="inlineStr">
+        <is>
+          <t>dthorne@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L122" s="4" t="inlineStr"/>
+      <c r="M122" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Frederick-MD-688/</t>
         </is>
@@ -7039,7 +7773,13 @@
         </is>
       </c>
       <c r="J123" s="4" t="inlineStr"/>
-      <c r="K123" s="3" t="inlineStr">
+      <c r="K123" s="4" t="inlineStr">
+        <is>
+          <t>tjohnson@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L123" s="4" t="inlineStr"/>
+      <c r="M123" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Forest-Hill-MD-3273/</t>
         </is>
@@ -7092,7 +7832,13 @@
         </is>
       </c>
       <c r="J124" s="4" t="inlineStr"/>
-      <c r="K124" s="3" t="inlineStr">
+      <c r="K124" s="4" t="inlineStr">
+        <is>
+          <t>skwak@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L124" s="4" t="inlineStr"/>
+      <c r="M124" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Gaithersburg-MD-3206/</t>
         </is>
@@ -7145,7 +7891,17 @@
         </is>
       </c>
       <c r="J125" s="4" t="inlineStr"/>
-      <c r="K125" s="3" t="inlineStr">
+      <c r="K125" s="4" t="inlineStr">
+        <is>
+          <t>rmarai@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L125" s="4" t="inlineStr">
+        <is>
+          <t>mtasleem@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M125" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Silver-Spring-MD-3274/</t>
         </is>
@@ -7198,7 +7954,13 @@
         </is>
       </c>
       <c r="J126" s="4" t="inlineStr"/>
-      <c r="K126" s="3" t="inlineStr">
+      <c r="K126" s="4" t="inlineStr">
+        <is>
+          <t>dfrench@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L126" s="4" t="inlineStr"/>
+      <c r="M126" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Portland-ME-560/</t>
         </is>
@@ -7255,7 +8017,9 @@
           <t>dvansickle@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K127" s="3" t="inlineStr">
+      <c r="K127" s="4" t="inlineStr"/>
+      <c r="L127" s="4" t="inlineStr"/>
+      <c r="M127" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Sterling-Heights-MI-580/</t>
         </is>
@@ -7304,7 +8068,9 @@
           <t>adabrowski@fishwindowcleaning.com; blang@fishwindowcleaning.com; dvansickle@fishwindowcleaning.com; hemang@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K128" s="3" t="inlineStr">
+      <c r="K128" s="4" t="inlineStr"/>
+      <c r="L128" s="4" t="inlineStr"/>
+      <c r="M128" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Detroit/</t>
         </is>
@@ -7357,7 +8123,13 @@
         </is>
       </c>
       <c r="J129" s="4" t="inlineStr"/>
-      <c r="K129" s="3" t="inlineStr">
+      <c r="K129" s="4" t="inlineStr">
+        <is>
+          <t>rcross@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L129" s="4" t="inlineStr"/>
+      <c r="M129" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Grand-Rapids-MI-460/</t>
         </is>
@@ -7410,7 +8182,17 @@
         </is>
       </c>
       <c r="J130" s="4" t="inlineStr"/>
-      <c r="K130" s="3" t="inlineStr">
+      <c r="K130" s="4" t="inlineStr">
+        <is>
+          <t>kbrown@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L130" s="4" t="inlineStr">
+        <is>
+          <t>nbrown@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M130" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Kalamazoo-MI-647/</t>
         </is>
@@ -7463,7 +8245,17 @@
         </is>
       </c>
       <c r="J131" s="4" t="inlineStr"/>
-      <c r="K131" s="3" t="inlineStr">
+      <c r="K131" s="4" t="inlineStr">
+        <is>
+          <t>abessinger@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L131" s="4" t="inlineStr">
+        <is>
+          <t>kbessinger@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M131" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Muskegon-MI-862/</t>
         </is>
@@ -7516,7 +8308,17 @@
         </is>
       </c>
       <c r="J132" s="4" t="inlineStr"/>
-      <c r="K132" s="3" t="inlineStr">
+      <c r="K132" s="4" t="inlineStr">
+        <is>
+          <t>jcullen@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L132" s="4" t="inlineStr">
+        <is>
+          <t>ceberhart@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M132" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Lansing-MI-883/</t>
         </is>
@@ -7573,7 +8375,9 @@
           <t>hemang@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K133" s="3" t="inlineStr">
+      <c r="K133" s="4" t="inlineStr"/>
+      <c r="L133" s="4" t="inlineStr"/>
+      <c r="M133" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Livonia-MI-678/</t>
         </is>
@@ -7630,7 +8434,9 @@
           <t>adabrowski@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K134" s="3" t="inlineStr">
+      <c r="K134" s="4" t="inlineStr"/>
+      <c r="L134" s="4" t="inlineStr"/>
+      <c r="M134" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Detroit-MI-3207/</t>
         </is>
@@ -7683,7 +8489,17 @@
         </is>
       </c>
       <c r="J135" s="4" t="inlineStr"/>
-      <c r="K135" s="3" t="inlineStr">
+      <c r="K135" s="4" t="inlineStr">
+        <is>
+          <t>kinbody@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L135" s="4" t="inlineStr">
+        <is>
+          <t>jsteiner@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M135" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Traverse-City-MI-290/</t>
         </is>
@@ -7740,7 +8556,9 @@
           <t>blang@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K136" s="3" t="inlineStr">
+      <c r="K136" s="4" t="inlineStr"/>
+      <c r="L136" s="4" t="inlineStr"/>
+      <c r="M136" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Detroit-MI-540/</t>
         </is>
@@ -7797,7 +8615,9 @@
           <t>kirkstensrud@gmail.com</t>
         </is>
       </c>
-      <c r="K137" s="3" t="inlineStr">
+      <c r="K137" s="4" t="inlineStr"/>
+      <c r="L137" s="4" t="inlineStr"/>
+      <c r="M137" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Eden-Prairie-MN-315/</t>
         </is>
@@ -7846,7 +8666,9 @@
           <t>arucker@fishwindowcleaning.com; kirkstensrud@gmail.com; mkern@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K138" s="3" t="inlineStr">
+      <c r="K138" s="4" t="inlineStr"/>
+      <c r="L138" s="4" t="inlineStr"/>
+      <c r="M138" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Minneapolis/</t>
         </is>
@@ -7903,7 +8725,9 @@
           <t>mkern@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K139" s="3" t="inlineStr">
+      <c r="K139" s="4" t="inlineStr"/>
+      <c r="L139" s="4" t="inlineStr"/>
+      <c r="M139" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Northwest-Twin-Cities-MN-3275/</t>
         </is>
@@ -7960,7 +8784,9 @@
           <t>arucker@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K140" s="3" t="inlineStr">
+      <c r="K140" s="4" t="inlineStr"/>
+      <c r="L140" s="4" t="inlineStr"/>
+      <c r="M140" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Saint-Paul-MN-863/</t>
         </is>
@@ -8017,7 +8843,9 @@
           <t>arucker@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K141" s="3" t="inlineStr">
+      <c r="K141" s="4" t="inlineStr"/>
+      <c r="L141" s="4" t="inlineStr"/>
+      <c r="M141" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Saint-Paul-MN-3182/</t>
         </is>
@@ -8070,7 +8898,13 @@
         </is>
       </c>
       <c r="J142" s="4" t="inlineStr"/>
-      <c r="K142" s="3" t="inlineStr">
+      <c r="K142" s="4" t="inlineStr">
+        <is>
+          <t>ahibbler@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L142" s="4" t="inlineStr"/>
+      <c r="M142" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Florissant-MO-671/</t>
         </is>
@@ -8119,7 +8953,9 @@
           <t>jallin@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K143" s="3" t="inlineStr">
+      <c r="K143" s="4" t="inlineStr"/>
+      <c r="L143" s="4" t="inlineStr"/>
+      <c r="M143" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/KansasCity/</t>
         </is>
@@ -8176,7 +9012,9 @@
           <t>jallin@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K144" s="3" t="inlineStr">
+      <c r="K144" s="4" t="inlineStr"/>
+      <c r="L144" s="4" t="inlineStr"/>
+      <c r="M144" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/KCMO/</t>
         </is>
@@ -8209,7 +9047,9 @@
         </is>
       </c>
       <c r="J145" s="4" t="inlineStr"/>
-      <c r="K145" s="3" t="inlineStr">
+      <c r="K145" s="4" t="inlineStr"/>
+      <c r="L145" s="4" t="inlineStr"/>
+      <c r="M145" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/1/</t>
         </is>
@@ -8262,7 +9102,13 @@
         </is>
       </c>
       <c r="J146" s="4" t="inlineStr"/>
-      <c r="K146" s="3" t="inlineStr">
+      <c r="K146" s="4" t="inlineStr">
+        <is>
+          <t>jcarroll@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L146" s="4" t="inlineStr"/>
+      <c r="M146" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/St-Louis-MO-3255/</t>
         </is>
@@ -8315,7 +9161,17 @@
         </is>
       </c>
       <c r="J147" s="4" t="inlineStr"/>
-      <c r="K147" s="3" t="inlineStr">
+      <c r="K147" s="4" t="inlineStr">
+        <is>
+          <t>vverdoorn@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L147" s="4" t="inlineStr">
+        <is>
+          <t>lverdoorn@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M147" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Springfield-MO-3262/</t>
         </is>
@@ -8368,7 +9224,13 @@
         </is>
       </c>
       <c r="J148" s="4" t="inlineStr"/>
-      <c r="K148" s="3" t="inlineStr">
+      <c r="K148" s="4" t="inlineStr">
+        <is>
+          <t>bfiala@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L148" s="4" t="inlineStr"/>
+      <c r="M148" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/St-Charles-MO-545/</t>
         </is>
@@ -8421,7 +9283,13 @@
         </is>
       </c>
       <c r="J149" s="4" t="inlineStr"/>
-      <c r="K149" s="3" t="inlineStr">
+      <c r="K149" s="4" t="inlineStr">
+        <is>
+          <t>mmerrick@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L149" s="4" t="inlineStr"/>
+      <c r="M149" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/St-Louis-MO-2/</t>
         </is>
@@ -8474,7 +9342,13 @@
         </is>
       </c>
       <c r="J150" s="4" t="inlineStr"/>
-      <c r="K150" s="3" t="inlineStr">
+      <c r="K150" s="4" t="inlineStr">
+        <is>
+          <t>tschwab@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L150" s="4" t="inlineStr"/>
+      <c r="M150" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Billings-MT-673/</t>
         </is>
@@ -8527,7 +9401,13 @@
         </is>
       </c>
       <c r="J151" s="4" t="inlineStr"/>
-      <c r="K151" s="3" t="inlineStr">
+      <c r="K151" s="4" t="inlineStr">
+        <is>
+          <t>ktreece@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L151" s="4" t="inlineStr"/>
+      <c r="M151" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Missoula-MT-3170/</t>
         </is>
@@ -8580,7 +9460,17 @@
         </is>
       </c>
       <c r="J152" s="4" t="inlineStr"/>
-      <c r="K152" s="3" t="inlineStr">
+      <c r="K152" s="4" t="inlineStr">
+        <is>
+          <t>jhitmar@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L152" s="4" t="inlineStr">
+        <is>
+          <t>lhitmar@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M152" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Cary-Durham-NC-3024/</t>
         </is>
@@ -8633,7 +9523,13 @@
         </is>
       </c>
       <c r="J153" s="4" t="inlineStr"/>
-      <c r="K153" s="3" t="inlineStr">
+      <c r="K153" s="4" t="inlineStr">
+        <is>
+          <t>aadedeji@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L153" s="4" t="inlineStr"/>
+      <c r="M153" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Charlotte-Metro-West-NC-3296/</t>
         </is>
@@ -8686,7 +9582,13 @@
         </is>
       </c>
       <c r="J154" s="4" t="inlineStr"/>
-      <c r="K154" s="3" t="inlineStr">
+      <c r="K154" s="4" t="inlineStr">
+        <is>
+          <t>lfrerich@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L154" s="4" t="inlineStr"/>
+      <c r="M154" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Charlotte-NC-861/</t>
         </is>
@@ -8739,7 +9641,17 @@
         </is>
       </c>
       <c r="J155" s="4" t="inlineStr"/>
-      <c r="K155" s="3" t="inlineStr">
+      <c r="K155" s="4" t="inlineStr">
+        <is>
+          <t>efuge@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L155" s="4" t="inlineStr">
+        <is>
+          <t>dfuge@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M155" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Concord-NC-3081/</t>
         </is>
@@ -8792,7 +9704,13 @@
         </is>
       </c>
       <c r="J156" s="4" t="inlineStr"/>
-      <c r="K156" s="3" t="inlineStr">
+      <c r="K156" s="4" t="inlineStr">
+        <is>
+          <t>tmoses@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L156" s="4" t="inlineStr"/>
+      <c r="M156" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Fayetteville-NC-3211/</t>
         </is>
@@ -8845,7 +9763,13 @@
         </is>
       </c>
       <c r="J157" s="4" t="inlineStr"/>
-      <c r="K157" s="3" t="inlineStr">
+      <c r="K157" s="4" t="inlineStr">
+        <is>
+          <t>bvondohlen@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L157" s="4" t="inlineStr"/>
+      <c r="M157" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Greensboro-NC-648/</t>
         </is>
@@ -8898,7 +9822,13 @@
         </is>
       </c>
       <c r="J158" s="4" t="inlineStr"/>
-      <c r="K158" s="3" t="inlineStr">
+      <c r="K158" s="4" t="inlineStr">
+        <is>
+          <t>tcarter@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L158" s="4" t="inlineStr"/>
+      <c r="M158" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Greenville-NC-3252/</t>
         </is>
@@ -8951,7 +9881,17 @@
         </is>
       </c>
       <c r="J159" s="4" t="inlineStr"/>
-      <c r="K159" s="3" t="inlineStr">
+      <c r="K159" s="4" t="inlineStr">
+        <is>
+          <t>pbarufkin@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L159" s="4" t="inlineStr">
+        <is>
+          <t>hbarufkin@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M159" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Raleigh-NC-654/</t>
         </is>
@@ -9004,7 +9944,13 @@
         </is>
       </c>
       <c r="J160" s="4" t="inlineStr"/>
-      <c r="K160" s="3" t="inlineStr">
+      <c r="K160" s="4" t="inlineStr">
+        <is>
+          <t>bjohnson@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L160" s="4" t="inlineStr"/>
+      <c r="M160" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Lincoln-NE-845/</t>
         </is>
@@ -9057,7 +10003,13 @@
         </is>
       </c>
       <c r="J161" s="4" t="inlineStr"/>
-      <c r="K161" s="3" t="inlineStr">
+      <c r="K161" s="4" t="inlineStr">
+        <is>
+          <t>cdrew@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L161" s="4" t="inlineStr"/>
+      <c r="M161" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Omaha-NE-873/</t>
         </is>
@@ -9110,7 +10062,17 @@
         </is>
       </c>
       <c r="J162" s="4" t="inlineStr"/>
-      <c r="K162" s="3" t="inlineStr">
+      <c r="K162" s="4" t="inlineStr">
+        <is>
+          <t>mjohns@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L162" s="4" t="inlineStr">
+        <is>
+          <t>kjohns@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M162" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Concord-NH-3067/</t>
         </is>
@@ -9163,7 +10125,13 @@
         </is>
       </c>
       <c r="J163" s="4" t="inlineStr"/>
-      <c r="K163" s="3" t="inlineStr">
+      <c r="K163" s="4" t="inlineStr">
+        <is>
+          <t>pthurston@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L163" s="4" t="inlineStr"/>
+      <c r="M163" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Nashua-NH-385/</t>
         </is>
@@ -9212,7 +10180,13 @@
         </is>
       </c>
       <c r="J164" s="4" t="inlineStr"/>
-      <c r="K164" s="3" t="inlineStr">
+      <c r="K164" s="4" t="inlineStr">
+        <is>
+          <t>bdower@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L164" s="4" t="inlineStr"/>
+      <c r="M164" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Portsmouth-NH-30500/</t>
         </is>
@@ -9265,7 +10239,17 @@
         </is>
       </c>
       <c r="J165" s="4" t="inlineStr"/>
-      <c r="K165" s="3" t="inlineStr">
+      <c r="K165" s="4" t="inlineStr">
+        <is>
+          <t>wfulton@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L165" s="4" t="inlineStr">
+        <is>
+          <t>kfulton@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M165" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Camden-NJ-645/</t>
         </is>
@@ -9318,7 +10302,13 @@
         </is>
       </c>
       <c r="J166" s="4" t="inlineStr"/>
-      <c r="K166" s="3" t="inlineStr">
+      <c r="K166" s="4" t="inlineStr">
+        <is>
+          <t>rhewins@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L166" s="4" t="inlineStr"/>
+      <c r="M166" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Paramus-NJ-697/</t>
         </is>
@@ -9371,7 +10361,17 @@
         </is>
       </c>
       <c r="J167" s="4" t="inlineStr"/>
-      <c r="K167" s="3" t="inlineStr">
+      <c r="K167" s="4" t="inlineStr">
+        <is>
+          <t>eschafer@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L167" s="4" t="inlineStr">
+        <is>
+          <t>rschafer@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M167" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Freehold-NJ-683/</t>
         </is>
@@ -9424,7 +10424,17 @@
         </is>
       </c>
       <c r="J168" s="4" t="inlineStr"/>
-      <c r="K168" s="3" t="inlineStr">
+      <c r="K168" s="4" t="inlineStr">
+        <is>
+          <t>sboutsikaris@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L168" s="4" t="inlineStr">
+        <is>
+          <t>eboutsikaris@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M168" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Somerset-NJ-693/</t>
         </is>
@@ -9477,7 +10487,13 @@
         </is>
       </c>
       <c r="J169" s="4" t="inlineStr"/>
-      <c r="K169" s="3" t="inlineStr">
+      <c r="K169" s="4" t="inlineStr">
+        <is>
+          <t>mstoecklin@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L169" s="4" t="inlineStr"/>
+      <c r="M169" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/East-Brunswick-NJ-3154/</t>
         </is>
@@ -9530,7 +10546,13 @@
         </is>
       </c>
       <c r="J170" s="4" t="inlineStr"/>
-      <c r="K170" s="3" t="inlineStr">
+      <c r="K170" s="4" t="inlineStr">
+        <is>
+          <t>klarkin@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L170" s="4" t="inlineStr"/>
+      <c r="M170" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Trenton-NJ-669/</t>
         </is>
@@ -9583,7 +10605,17 @@
         </is>
       </c>
       <c r="J171" s="4" t="inlineStr"/>
-      <c r="K171" s="3" t="inlineStr">
+      <c r="K171" s="4" t="inlineStr">
+        <is>
+          <t>scuster@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L171" s="4" t="inlineStr">
+        <is>
+          <t>gcuster@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M171" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Las-Vegas-NV-3166/</t>
         </is>
@@ -9636,7 +10668,13 @@
         </is>
       </c>
       <c r="J172" s="4" t="inlineStr"/>
-      <c r="K172" s="3" t="inlineStr">
+      <c r="K172" s="4" t="inlineStr">
+        <is>
+          <t>kriley@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L172" s="4" t="inlineStr"/>
+      <c r="M172" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Sparks-NV-3278/</t>
         </is>
@@ -9689,7 +10727,17 @@
         </is>
       </c>
       <c r="J173" s="4" t="inlineStr"/>
-      <c r="K173" s="3" t="inlineStr">
+      <c r="K173" s="4" t="inlineStr">
+        <is>
+          <t>adasalla@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L173" s="4" t="inlineStr">
+        <is>
+          <t>bdasalla@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M173" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Nassau-County-NY-3298/</t>
         </is>
@@ -9742,7 +10790,13 @@
         </is>
       </c>
       <c r="J174" s="4" t="inlineStr"/>
-      <c r="K174" s="3" t="inlineStr">
+      <c r="K174" s="4" t="inlineStr">
+        <is>
+          <t>cschottland@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L174" s="4" t="inlineStr"/>
+      <c r="M174" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Rochester-NY-875/</t>
         </is>
@@ -9795,7 +10849,13 @@
         </is>
       </c>
       <c r="J175" s="4" t="inlineStr"/>
-      <c r="K175" s="3" t="inlineStr">
+      <c r="K175" s="4" t="inlineStr">
+        <is>
+          <t>msilverstein@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L175" s="4" t="inlineStr"/>
+      <c r="M175" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Fairfield-Westchester-6100/</t>
         </is>
@@ -9848,7 +10908,13 @@
         </is>
       </c>
       <c r="J176" s="4" t="inlineStr"/>
-      <c r="K176" s="3" t="inlineStr">
+      <c r="K176" s="4" t="inlineStr">
+        <is>
+          <t>kvansanford@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L176" s="4" t="inlineStr"/>
+      <c r="M176" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Syracuse-NY-3288/</t>
         </is>
@@ -9897,7 +10963,9 @@
           <t>phays@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K177" s="3" t="inlineStr">
+      <c r="K177" s="4" t="inlineStr"/>
+      <c r="L177" s="4" t="inlineStr"/>
+      <c r="M177" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Cleveland-OH-3201/</t>
         </is>
@@ -9954,7 +11022,9 @@
           <t>phays@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K178" s="3" t="inlineStr">
+      <c r="K178" s="4" t="inlineStr"/>
+      <c r="L178" s="4" t="inlineStr"/>
+      <c r="M178" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Akron-OH-684/</t>
         </is>
@@ -10003,7 +11073,9 @@
           <t>phays@fishwindowcleaning.com; pprucey@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K179" s="3" t="inlineStr">
+      <c r="K179" s="4" t="inlineStr"/>
+      <c r="L179" s="4" t="inlineStr"/>
+      <c r="M179" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Cleveland/</t>
         </is>
@@ -10056,7 +11128,13 @@
         </is>
       </c>
       <c r="J180" s="4" t="inlineStr"/>
-      <c r="K180" s="3" t="inlineStr">
+      <c r="K180" s="4" t="inlineStr">
+        <is>
+          <t>sjude@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L180" s="4" t="inlineStr"/>
+      <c r="M180" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Columbus-OH-890/</t>
         </is>
@@ -10109,7 +11187,13 @@
         </is>
       </c>
       <c r="J181" s="4" t="inlineStr"/>
-      <c r="K181" s="3" t="inlineStr">
+      <c r="K181" s="4" t="inlineStr">
+        <is>
+          <t>nsnelson@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L181" s="4" t="inlineStr"/>
+      <c r="M181" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Westerville-OH-3119/</t>
         </is>
@@ -10166,7 +11250,9 @@
           <t>pprucey@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K182" s="3" t="inlineStr">
+      <c r="K182" s="4" t="inlineStr"/>
+      <c r="L182" s="4" t="inlineStr"/>
+      <c r="M182" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Mentor-OH-3136/</t>
         </is>
@@ -10219,7 +11305,13 @@
         </is>
       </c>
       <c r="J183" s="4" t="inlineStr"/>
-      <c r="K183" s="3" t="inlineStr">
+      <c r="K183" s="4" t="inlineStr">
+        <is>
+          <t>meisenzimmer@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L183" s="4" t="inlineStr"/>
+      <c r="M183" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Akron-OH-3055/</t>
         </is>
@@ -10272,7 +11364,17 @@
         </is>
       </c>
       <c r="J184" s="4" t="inlineStr"/>
-      <c r="K184" s="3" t="inlineStr">
+      <c r="K184" s="4" t="inlineStr">
+        <is>
+          <t>tcarver@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L184" s="4" t="inlineStr">
+        <is>
+          <t>scarver@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M184" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/SW-Ohio-N-Kentucky-SE-Indiana-3044/</t>
         </is>
@@ -10325,7 +11427,17 @@
         </is>
       </c>
       <c r="J185" s="4" t="inlineStr"/>
-      <c r="K185" s="3" t="inlineStr">
+      <c r="K185" s="4" t="inlineStr">
+        <is>
+          <t>dmusteric@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L185" s="4" t="inlineStr">
+        <is>
+          <t>jmusteric@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M185" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Toledo-OH-665/</t>
         </is>
@@ -10378,7 +11490,17 @@
         </is>
       </c>
       <c r="J186" s="4" t="inlineStr"/>
-      <c r="K186" s="3" t="inlineStr">
+      <c r="K186" s="4" t="inlineStr">
+        <is>
+          <t>kstabi@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L186" s="4" t="inlineStr">
+        <is>
+          <t>jstabi@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M186" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Youngstown-OH-3210/</t>
         </is>
@@ -10431,7 +11553,17 @@
         </is>
       </c>
       <c r="J187" s="4" t="inlineStr"/>
-      <c r="K187" s="3" t="inlineStr">
+      <c r="K187" s="4" t="inlineStr">
+        <is>
+          <t>hriggins@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L187" s="4" t="inlineStr">
+        <is>
+          <t>lriggins@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M187" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Edmond-OK-3295/</t>
         </is>
@@ -10484,7 +11616,13 @@
         </is>
       </c>
       <c r="J188" s="4" t="inlineStr"/>
-      <c r="K188" s="3" t="inlineStr">
+      <c r="K188" s="4" t="inlineStr">
+        <is>
+          <t>gkelton@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L188" s="4" t="inlineStr"/>
+      <c r="M188" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Oklahoma-City-OK-3165/</t>
         </is>
@@ -10537,7 +11675,17 @@
         </is>
       </c>
       <c r="J189" s="4" t="inlineStr"/>
-      <c r="K189" s="3" t="inlineStr">
+      <c r="K189" s="4" t="inlineStr">
+        <is>
+          <t>klambert@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L189" s="4" t="inlineStr">
+        <is>
+          <t>plambert@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M189" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Beaverton-OR-633/</t>
         </is>
@@ -10590,7 +11738,17 @@
         </is>
       </c>
       <c r="J190" s="4" t="inlineStr"/>
-      <c r="K190" s="3" t="inlineStr">
+      <c r="K190" s="4" t="inlineStr">
+        <is>
+          <t>csweistris@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L190" s="4" t="inlineStr">
+        <is>
+          <t>dsweistris@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M190" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Bend-OR-613/</t>
         </is>
@@ -10643,7 +11801,13 @@
         </is>
       </c>
       <c r="J191" s="4" t="inlineStr"/>
-      <c r="K191" s="3" t="inlineStr">
+      <c r="K191" s="4" t="inlineStr">
+        <is>
+          <t>ldrouhard@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L191" s="4" t="inlineStr"/>
+      <c r="M191" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Corvallis-OR-3235/</t>
         </is>
@@ -10696,7 +11860,13 @@
         </is>
       </c>
       <c r="J192" s="4" t="inlineStr"/>
-      <c r="K192" s="3" t="inlineStr">
+      <c r="K192" s="4" t="inlineStr">
+        <is>
+          <t>dgalkin@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L192" s="4" t="inlineStr"/>
+      <c r="M192" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Allentown-PA-3110/</t>
         </is>
@@ -10749,7 +11919,13 @@
         </is>
       </c>
       <c r="J193" s="4" t="inlineStr"/>
-      <c r="K193" s="3" t="inlineStr">
+      <c r="K193" s="4" t="inlineStr">
+        <is>
+          <t>lbaehr@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L193" s="4" t="inlineStr"/>
+      <c r="M193" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Butler-PA-3117/</t>
         </is>
@@ -10802,7 +11978,17 @@
         </is>
       </c>
       <c r="J194" s="4" t="inlineStr"/>
-      <c r="K194" s="3" t="inlineStr">
+      <c r="K194" s="4" t="inlineStr">
+        <is>
+          <t>kkeller@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L194" s="4" t="inlineStr">
+        <is>
+          <t>gkeller@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M194" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Harrisburg-PA-720/</t>
         </is>
@@ -10855,7 +12041,17 @@
         </is>
       </c>
       <c r="J195" s="4" t="inlineStr"/>
-      <c r="K195" s="3" t="inlineStr">
+      <c r="K195" s="4" t="inlineStr">
+        <is>
+          <t>qhartman@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L195" s="4" t="inlineStr">
+        <is>
+          <t>shartman@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M195" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Lancaster-PA-3113/</t>
         </is>
@@ -10908,7 +12104,17 @@
         </is>
       </c>
       <c r="J196" s="4" t="inlineStr"/>
-      <c r="K196" s="3" t="inlineStr">
+      <c r="K196" s="4" t="inlineStr">
+        <is>
+          <t>ryoung@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L196" s="4" t="inlineStr">
+        <is>
+          <t>byoung@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M196" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Norristown-PA-670/</t>
         </is>
@@ -10961,7 +12167,13 @@
         </is>
       </c>
       <c r="J197" s="4" t="inlineStr"/>
-      <c r="K197" s="3" t="inlineStr">
+      <c r="K197" s="4" t="inlineStr">
+        <is>
+          <t>dgalkin@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L197" s="4" t="inlineStr"/>
+      <c r="M197" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Bensalem-PA-3008/</t>
         </is>
@@ -11014,7 +12226,17 @@
         </is>
       </c>
       <c r="J198" s="4" t="inlineStr"/>
-      <c r="K198" s="3" t="inlineStr">
+      <c r="K198" s="4" t="inlineStr">
+        <is>
+          <t>bschubert@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L198" s="4" t="inlineStr">
+        <is>
+          <t>aschubert@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M198" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Pittsburgh-PA-3115/</t>
         </is>
@@ -11067,7 +12289,13 @@
         </is>
       </c>
       <c r="J199" s="4" t="inlineStr"/>
-      <c r="K199" s="3" t="inlineStr">
+      <c r="K199" s="4" t="inlineStr">
+        <is>
+          <t>smcnaught@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L199" s="4" t="inlineStr"/>
+      <c r="M199" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Pittsburgh-PA-652/</t>
         </is>
@@ -11120,7 +12348,17 @@
         </is>
       </c>
       <c r="J200" s="4" t="inlineStr"/>
-      <c r="K200" s="3" t="inlineStr">
+      <c r="K200" s="4" t="inlineStr">
+        <is>
+          <t>cbommer@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L200" s="4" t="inlineStr">
+        <is>
+          <t>mbommer@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M200" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Pittsburgh-PA-3116/</t>
         </is>
@@ -11173,7 +12411,13 @@
         </is>
       </c>
       <c r="J201" s="4" t="inlineStr"/>
-      <c r="K201" s="3" t="inlineStr">
+      <c r="K201" s="4" t="inlineStr">
+        <is>
+          <t>jbuske@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L201" s="4" t="inlineStr"/>
+      <c r="M201" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/State-College-PA-3135/</t>
         </is>
@@ -11226,7 +12470,17 @@
         </is>
       </c>
       <c r="J202" s="4" t="inlineStr"/>
-      <c r="K202" s="3" t="inlineStr">
+      <c r="K202" s="4" t="inlineStr">
+        <is>
+          <t>ryoung@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L202" s="4" t="inlineStr">
+        <is>
+          <t>byoung@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M202" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/West-Chester-PA-3041/</t>
         </is>
@@ -11279,7 +12533,13 @@
         </is>
       </c>
       <c r="J203" s="4" t="inlineStr"/>
-      <c r="K203" s="3" t="inlineStr">
+      <c r="K203" s="4" t="inlineStr">
+        <is>
+          <t>dcotter@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L203" s="4" t="inlineStr"/>
+      <c r="M203" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Providence-RI-765/</t>
         </is>
@@ -11332,7 +12592,13 @@
         </is>
       </c>
       <c r="J204" s="4" t="inlineStr"/>
-      <c r="K204" s="3" t="inlineStr">
+      <c r="K204" s="4" t="inlineStr">
+        <is>
+          <t>tfinley@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L204" s="4" t="inlineStr"/>
+      <c r="M204" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Myrtle-Beach-SC-3068/</t>
         </is>
@@ -11385,7 +12651,13 @@
         </is>
       </c>
       <c r="J205" s="4" t="inlineStr"/>
-      <c r="K205" s="3" t="inlineStr">
+      <c r="K205" s="4" t="inlineStr">
+        <is>
+          <t>dbryant@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L205" s="4" t="inlineStr"/>
+      <c r="M205" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Rock-Hill-SC-3248/</t>
         </is>
@@ -11438,7 +12710,13 @@
         </is>
       </c>
       <c r="J206" s="4" t="inlineStr"/>
-      <c r="K206" s="3" t="inlineStr">
+      <c r="K206" s="4" t="inlineStr">
+        <is>
+          <t>szumstein@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L206" s="4" t="inlineStr"/>
+      <c r="M206" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Charleston-SC-3283/</t>
         </is>
@@ -11491,7 +12769,13 @@
         </is>
       </c>
       <c r="J207" s="4" t="inlineStr"/>
-      <c r="K207" s="3" t="inlineStr">
+      <c r="K207" s="4" t="inlineStr">
+        <is>
+          <t>kjones@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L207" s="4" t="inlineStr"/>
+      <c r="M207" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Spartanburg-SC-3294/</t>
         </is>
@@ -11544,7 +12828,13 @@
         </is>
       </c>
       <c r="J208" s="4" t="inlineStr"/>
-      <c r="K208" s="3" t="inlineStr">
+      <c r="K208" s="4" t="inlineStr">
+        <is>
+          <t>bteachout@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L208" s="4" t="inlineStr"/>
+      <c r="M208" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Rapid-City-SD-679/</t>
         </is>
@@ -11597,7 +12887,13 @@
         </is>
       </c>
       <c r="J209" s="4" t="inlineStr"/>
-      <c r="K209" s="3" t="inlineStr">
+      <c r="K209" s="4" t="inlineStr">
+        <is>
+          <t>ghale@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L209" s="4" t="inlineStr"/>
+      <c r="M209" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Johnson-City-TN-664/</t>
         </is>
@@ -11650,7 +12946,13 @@
         </is>
       </c>
       <c r="J210" s="4" t="inlineStr"/>
-      <c r="K210" s="3" t="inlineStr">
+      <c r="K210" s="4" t="inlineStr">
+        <is>
+          <t>jrandazzo@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L210" s="4" t="inlineStr"/>
+      <c r="M210" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Knoxville-TN-455/</t>
         </is>
@@ -11703,7 +13005,13 @@
         </is>
       </c>
       <c r="J211" s="4" t="inlineStr"/>
-      <c r="K211" s="3" t="inlineStr">
+      <c r="K211" s="4" t="inlineStr">
+        <is>
+          <t>jshannon@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L211" s="4" t="inlineStr"/>
+      <c r="M211" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Memphis-TN-3240/</t>
         </is>
@@ -11756,7 +13064,13 @@
         </is>
       </c>
       <c r="J212" s="4" t="inlineStr"/>
-      <c r="K212" s="3" t="inlineStr">
+      <c r="K212" s="4" t="inlineStr">
+        <is>
+          <t>jpedro@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L212" s="4" t="inlineStr"/>
+      <c r="M212" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Chattanooga-TN-3293/</t>
         </is>
@@ -11809,7 +13123,17 @@
         </is>
       </c>
       <c r="J213" s="4" t="inlineStr"/>
-      <c r="K213" s="3" t="inlineStr">
+      <c r="K213" s="4" t="inlineStr">
+        <is>
+          <t>drenwick@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L213" s="4" t="inlineStr">
+        <is>
+          <t>rrenwick@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M213" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Nashville-TN-625/</t>
         </is>
@@ -11862,7 +13186,13 @@
         </is>
       </c>
       <c r="J214" s="4" t="inlineStr"/>
-      <c r="K214" s="3" t="inlineStr">
+      <c r="K214" s="4" t="inlineStr">
+        <is>
+          <t>sesparza@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L214" s="4" t="inlineStr"/>
+      <c r="M214" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Austin-TX-440/</t>
         </is>
@@ -11915,7 +13245,17 @@
         </is>
       </c>
       <c r="J215" s="4" t="inlineStr"/>
-      <c r="K215" s="3" t="inlineStr">
+      <c r="K215" s="4" t="inlineStr">
+        <is>
+          <t>amaisonneuve@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L215" s="4" t="inlineStr">
+        <is>
+          <t>bmaisonneuve@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M215" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Beaumont-TX-657/</t>
         </is>
@@ -11968,7 +13308,13 @@
         </is>
       </c>
       <c r="J216" s="4" t="inlineStr"/>
-      <c r="K216" s="3" t="inlineStr">
+      <c r="K216" s="4" t="inlineStr">
+        <is>
+          <t>jnewton@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L216" s="4" t="inlineStr"/>
+      <c r="M216" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/College-Station-TX-821/</t>
         </is>
@@ -12021,7 +13367,13 @@
         </is>
       </c>
       <c r="J217" s="4" t="inlineStr"/>
-      <c r="K217" s="3" t="inlineStr">
+      <c r="K217" s="4" t="inlineStr">
+        <is>
+          <t>tgroseclose@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L217" s="4" t="inlineStr"/>
+      <c r="M217" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Corpus-Christi-TX-3133/</t>
         </is>
@@ -12078,7 +13430,9 @@
           <t>jcarswell@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K218" s="3" t="inlineStr">
+      <c r="K218" s="4" t="inlineStr"/>
+      <c r="L218" s="4" t="inlineStr"/>
+      <c r="M218" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Dallas-TX-2270/</t>
         </is>
@@ -12127,7 +13481,9 @@
           <t>esilver@fishwindowcleaning.com; jcarswell@fishwindowcleaning.com; lchadwick@fishwindowcleaning.com; pkoele@fishwindowcleaning.com; schastain@fishwindowcleaning.com; wwilliams@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K219" s="3" t="inlineStr">
+      <c r="K219" s="4" t="inlineStr"/>
+      <c r="L219" s="4" t="inlineStr"/>
+      <c r="M219" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/dfw/</t>
         </is>
@@ -12184,7 +13540,9 @@
           <t>pkoele@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K220" s="3" t="inlineStr">
+      <c r="K220" s="4" t="inlineStr"/>
+      <c r="L220" s="4" t="inlineStr"/>
+      <c r="M220" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Denton-TX-614/</t>
         </is>
@@ -12241,7 +13599,9 @@
           <t>lchadwick@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K221" s="3" t="inlineStr">
+      <c r="K221" s="4" t="inlineStr"/>
+      <c r="L221" s="4" t="inlineStr"/>
+      <c r="M221" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/DeSoto-TX-638/</t>
         </is>
@@ -12294,7 +13654,9 @@
         </is>
       </c>
       <c r="J222" s="4" t="inlineStr"/>
-      <c r="K222" s="3" t="inlineStr">
+      <c r="K222" s="4" t="inlineStr"/>
+      <c r="L222" s="4" t="inlineStr"/>
+      <c r="M222" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/tarrant/</t>
         </is>
@@ -12351,7 +13713,9 @@
           <t>esilver@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K223" s="3" t="inlineStr">
+      <c r="K223" s="4" t="inlineStr"/>
+      <c r="L223" s="4" t="inlineStr"/>
+      <c r="M223" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Fort-Worth-TX-637/</t>
         </is>
@@ -12408,7 +13772,9 @@
           <t>tallen@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K224" s="3" t="inlineStr">
+      <c r="K224" s="4" t="inlineStr"/>
+      <c r="L224" s="4" t="inlineStr"/>
+      <c r="M224" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Houston-TX-837/</t>
         </is>
@@ -12465,7 +13831,9 @@
           <t>jbassett@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K225" s="3" t="inlineStr">
+      <c r="K225" s="4" t="inlineStr"/>
+      <c r="L225" s="4" t="inlineStr"/>
+      <c r="M225" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Houston-TX-851/</t>
         </is>
@@ -12522,7 +13890,9 @@
           <t>tweissman@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K226" s="3" t="inlineStr">
+      <c r="K226" s="4" t="inlineStr"/>
+      <c r="L226" s="4" t="inlineStr"/>
+      <c r="M226" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Houston-TX-619/</t>
         </is>
@@ -12579,7 +13949,9 @@
           <t>ajohnson@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K227" s="3" t="inlineStr">
+      <c r="K227" s="4" t="inlineStr"/>
+      <c r="L227" s="4" t="inlineStr"/>
+      <c r="M227" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Houston-TX-3284/</t>
         </is>
@@ -12628,7 +14000,9 @@
           <t>ajohnson@fishwindowcleaning.com; jbassett@fishwindowcleaning.com; mjones@fishwindowcleaning.com; tallen@fishwindowcleaning.com; trentpeneston@fishwindowcleaning.com; tweissman@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K228" s="3" t="inlineStr">
+      <c r="K228" s="4" t="inlineStr"/>
+      <c r="L228" s="4" t="inlineStr"/>
+      <c r="M228" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Houston/</t>
         </is>
@@ -12685,7 +14059,9 @@
           <t>mjones@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K229" s="3" t="inlineStr">
+      <c r="K229" s="4" t="inlineStr"/>
+      <c r="L229" s="4" t="inlineStr"/>
+      <c r="M229" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Houston-TX-843/</t>
         </is>
@@ -12738,7 +14114,17 @@
         </is>
       </c>
       <c r="J230" s="4" t="inlineStr"/>
-      <c r="K230" s="3" t="inlineStr">
+      <c r="K230" s="4" t="inlineStr">
+        <is>
+          <t>jwilliamson@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L230" s="4" t="inlineStr">
+        <is>
+          <t>ewilliamson@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M230" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Killeen-TX-3238/</t>
         </is>
@@ -12795,7 +14181,9 @@
           <t>trentpeneston@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K231" s="3" t="inlineStr">
+      <c r="K231" s="4" t="inlineStr"/>
+      <c r="L231" s="4" t="inlineStr"/>
+      <c r="M231" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Conroe-TX-3009/</t>
         </is>
@@ -12852,7 +14240,9 @@
           <t>esilver@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K232" s="3" t="inlineStr">
+      <c r="K232" s="4" t="inlineStr"/>
+      <c r="L232" s="4" t="inlineStr"/>
+      <c r="M232" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Arlington-TX-855/</t>
         </is>
@@ -12905,7 +14295,17 @@
         </is>
       </c>
       <c r="J233" s="4" t="inlineStr"/>
-      <c r="K233" s="3" t="inlineStr">
+      <c r="K233" s="4" t="inlineStr">
+        <is>
+          <t>dhouse@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L233" s="4" t="inlineStr">
+        <is>
+          <t>ghouse@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M233" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/New-Braunfels-TX-3140/</t>
         </is>
@@ -12962,7 +14362,9 @@
           <t>schastain@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K234" s="3" t="inlineStr">
+      <c r="K234" s="4" t="inlineStr"/>
+      <c r="L234" s="4" t="inlineStr"/>
+      <c r="M234" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Garland-TX-895/</t>
         </is>
@@ -13015,7 +14417,17 @@
         </is>
       </c>
       <c r="J235" s="4" t="inlineStr"/>
-      <c r="K235" s="3" t="inlineStr">
+      <c r="K235" s="4" t="inlineStr">
+        <is>
+          <t>cguess@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L235" s="4" t="inlineStr">
+        <is>
+          <t>gguess@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M235" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/San-Antonio-TX-75/</t>
         </is>
@@ -13072,7 +14484,9 @@
           <t>wwilliams@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K236" s="3" t="inlineStr">
+      <c r="K236" s="4" t="inlineStr"/>
+      <c r="L236" s="4" t="inlineStr"/>
+      <c r="M236" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Arlington-TX-860/</t>
         </is>
@@ -13125,7 +14539,13 @@
         </is>
       </c>
       <c r="J237" s="4" t="inlineStr"/>
-      <c r="K237" s="3" t="inlineStr">
+      <c r="K237" s="4" t="inlineStr">
+        <is>
+          <t>bsilverstein@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L237" s="4" t="inlineStr"/>
+      <c r="M237" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Tyler-TX-3286/</t>
         </is>
@@ -13178,7 +14598,13 @@
         </is>
       </c>
       <c r="J238" s="4" t="inlineStr"/>
-      <c r="K238" s="3" t="inlineStr">
+      <c r="K238" s="4" t="inlineStr">
+        <is>
+          <t>dmills@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L238" s="4" t="inlineStr"/>
+      <c r="M238" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Waco-TX-3281/</t>
         </is>
@@ -13231,7 +14657,13 @@
         </is>
       </c>
       <c r="J239" s="4" t="inlineStr"/>
-      <c r="K239" s="3" t="inlineStr">
+      <c r="K239" s="4" t="inlineStr">
+        <is>
+          <t>award@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L239" s="4" t="inlineStr"/>
+      <c r="M239" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Salt-Lake-City-UT-857/</t>
         </is>
@@ -13284,7 +14716,13 @@
         </is>
       </c>
       <c r="J240" s="4" t="inlineStr"/>
-      <c r="K240" s="3" t="inlineStr">
+      <c r="K240" s="4" t="inlineStr">
+        <is>
+          <t>jfarhi@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L240" s="4" t="inlineStr"/>
+      <c r="M240" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Charlottesville-VA-3195/</t>
         </is>
@@ -13337,7 +14775,13 @@
         </is>
       </c>
       <c r="J241" s="4" t="inlineStr"/>
-      <c r="K241" s="3" t="inlineStr">
+      <c r="K241" s="4" t="inlineStr">
+        <is>
+          <t>cjohnson@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L241" s="4" t="inlineStr"/>
+      <c r="M241" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Fairfax-VA-3141/</t>
         </is>
@@ -13390,7 +14834,13 @@
         </is>
       </c>
       <c r="J242" s="4" t="inlineStr"/>
-      <c r="K242" s="3" t="inlineStr">
+      <c r="K242" s="4" t="inlineStr">
+        <is>
+          <t>mfaulkner@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L242" s="4" t="inlineStr"/>
+      <c r="M242" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Fredericksburg-VA-644/</t>
         </is>
@@ -13443,7 +14893,13 @@
         </is>
       </c>
       <c r="J243" s="4" t="inlineStr"/>
-      <c r="K243" s="3" t="inlineStr">
+      <c r="K243" s="4" t="inlineStr">
+        <is>
+          <t>lbryan@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L243" s="4" t="inlineStr"/>
+      <c r="M243" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Manassas-VA-3267/</t>
         </is>
@@ -13496,7 +14952,13 @@
         </is>
       </c>
       <c r="J244" s="4" t="inlineStr"/>
-      <c r="K244" s="3" t="inlineStr">
+      <c r="K244" s="4" t="inlineStr">
+        <is>
+          <t>jfarhi@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L244" s="4" t="inlineStr"/>
+      <c r="M244" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Richmond-VA-699/</t>
         </is>
@@ -13549,7 +15011,17 @@
         </is>
       </c>
       <c r="J245" s="4" t="inlineStr"/>
-      <c r="K245" s="3" t="inlineStr">
+      <c r="K245" s="4" t="inlineStr">
+        <is>
+          <t>rrowe@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L245" s="4" t="inlineStr">
+        <is>
+          <t>ibratianu@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M245" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Virginia-Beach-VA-535/</t>
         </is>
@@ -13602,7 +15074,13 @@
         </is>
       </c>
       <c r="J246" s="4" t="inlineStr"/>
-      <c r="K246" s="3" t="inlineStr">
+      <c r="K246" s="4" t="inlineStr">
+        <is>
+          <t>aforet@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L246" s="4" t="inlineStr"/>
+      <c r="M246" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Williamsburg-VA-3109/</t>
         </is>
@@ -13655,7 +15133,13 @@
         </is>
       </c>
       <c r="J247" s="4" t="inlineStr"/>
-      <c r="K247" s="3" t="inlineStr">
+      <c r="K247" s="4" t="inlineStr">
+        <is>
+          <t>mholman@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L247" s="4" t="inlineStr"/>
+      <c r="M247" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Bellevue-WA-694/</t>
         </is>
@@ -13708,7 +15192,17 @@
         </is>
       </c>
       <c r="J248" s="4" t="inlineStr"/>
-      <c r="K248" s="3" t="inlineStr">
+      <c r="K248" s="4" t="inlineStr">
+        <is>
+          <t>pboisseau@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L248" s="4" t="inlineStr">
+        <is>
+          <t>jboisseau@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M248" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Kent-WA-3282/</t>
         </is>
@@ -13761,7 +15255,13 @@
         </is>
       </c>
       <c r="J249" s="4" t="inlineStr"/>
-      <c r="K249" s="3" t="inlineStr">
+      <c r="K249" s="4" t="inlineStr">
+        <is>
+          <t>gnixon@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L249" s="4" t="inlineStr"/>
+      <c r="M249" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Spokane-WA-3097/</t>
         </is>
@@ -13814,7 +15314,17 @@
         </is>
       </c>
       <c r="J250" s="4" t="inlineStr"/>
-      <c r="K250" s="3" t="inlineStr">
+      <c r="K250" s="4" t="inlineStr">
+        <is>
+          <t>rstanfill@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L250" s="4" t="inlineStr">
+        <is>
+          <t>cstanfill@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M250" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Vancouver-WA-634/</t>
         </is>
@@ -13871,7 +15381,9 @@
           <t>cstraka@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K251" s="3" t="inlineStr">
+      <c r="K251" s="4" t="inlineStr"/>
+      <c r="L251" s="4" t="inlineStr"/>
+      <c r="M251" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Burlington-WI-3063/</t>
         </is>
@@ -13924,7 +15436,13 @@
         </is>
       </c>
       <c r="J252" s="4" t="inlineStr"/>
-      <c r="K252" s="3" t="inlineStr">
+      <c r="K252" s="4" t="inlineStr">
+        <is>
+          <t>tespeseth@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L252" s="4" t="inlineStr"/>
+      <c r="M252" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Eau-Claire-WI-775/</t>
         </is>
@@ -13977,7 +15495,13 @@
         </is>
       </c>
       <c r="J253" s="4" t="inlineStr"/>
-      <c r="K253" s="3" t="inlineStr">
+      <c r="K253" s="4" t="inlineStr">
+        <is>
+          <t>charing@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L253" s="4" t="inlineStr"/>
+      <c r="M253" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Appleton-Green-Bay-WI-680/</t>
         </is>
@@ -14030,7 +15554,17 @@
         </is>
       </c>
       <c r="J254" s="4" t="inlineStr"/>
-      <c r="K254" s="3" t="inlineStr">
+      <c r="K254" s="4" t="inlineStr">
+        <is>
+          <t>jspude@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L254" s="4" t="inlineStr">
+        <is>
+          <t>dspude@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M254" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Janesville-WI-3064/</t>
         </is>
@@ -14083,7 +15617,17 @@
         </is>
       </c>
       <c r="J255" s="4" t="inlineStr"/>
-      <c r="K255" s="3" t="inlineStr">
+      <c r="K255" s="4" t="inlineStr">
+        <is>
+          <t>cgilding@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L255" s="4" t="inlineStr">
+        <is>
+          <t>bgilding@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="M255" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Madison-WI-626/</t>
         </is>
@@ -14132,7 +15676,9 @@
           <t>gcurtis@fishwindowcleaning.com; ntraverse@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K256" s="3" t="inlineStr">
+      <c r="K256" s="4" t="inlineStr"/>
+      <c r="L256" s="4" t="inlineStr"/>
+      <c r="M256" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Milwaukee/</t>
         </is>
@@ -14189,7 +15735,9 @@
           <t>ntraverse@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K257" s="3" t="inlineStr">
+      <c r="K257" s="4" t="inlineStr"/>
+      <c r="L257" s="4" t="inlineStr"/>
+      <c r="M257" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Milwaukee-WI-864/</t>
         </is>
@@ -14246,7 +15794,9 @@
           <t>gcurtis@fishwindowcleaning.com</t>
         </is>
       </c>
-      <c r="K258" s="3" t="inlineStr">
+      <c r="K258" s="4" t="inlineStr"/>
+      <c r="L258" s="4" t="inlineStr"/>
+      <c r="M258" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Milwaukee-WI-663/</t>
         </is>
@@ -14299,7 +15849,13 @@
         </is>
       </c>
       <c r="J259" s="4" t="inlineStr"/>
-      <c r="K259" s="3" t="inlineStr">
+      <c r="K259" s="4" t="inlineStr">
+        <is>
+          <t>charing@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L259" s="4" t="inlineStr"/>
+      <c r="M259" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Wausau-WI-3186/</t>
         </is>
@@ -14352,7 +15908,13 @@
         </is>
       </c>
       <c r="J260" s="4" t="inlineStr"/>
-      <c r="K260" s="3" t="inlineStr">
+      <c r="K260" s="4" t="inlineStr">
+        <is>
+          <t>qclark@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L260" s="4" t="inlineStr"/>
+      <c r="M260" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Casper-WY-3203/</t>
         </is>
@@ -14405,7 +15967,13 @@
         </is>
       </c>
       <c r="J261" s="4" t="inlineStr"/>
-      <c r="K261" s="3" t="inlineStr">
+      <c r="K261" s="4" t="inlineStr">
+        <is>
+          <t>mbarrett@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L261" s="4" t="inlineStr"/>
+      <c r="M261" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Cheyenne-WY-3290/</t>
         </is>
@@ -14458,14 +16026,20 @@
         </is>
       </c>
       <c r="J262" s="4" t="inlineStr"/>
-      <c r="K262" s="3" t="inlineStr">
+      <c r="K262" s="4" t="inlineStr">
+        <is>
+          <t>bteachout@fishwindowcleaning.com</t>
+        </is>
+      </c>
+      <c r="L262" s="4" t="inlineStr"/>
+      <c r="M262" s="3" t="inlineStr">
         <is>
           <t>https://www.fishwindowcleaning.com/Gillette-WY-6790/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K262"/>
+  <autoFilter ref="A1:M262"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14476,7 +16050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14568,10 +16142,34 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
+          <t>Likely Email</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>NOT published anywhere on the site. Built from the corporate pattern first initial + last name @fishwindowcleaning.com (e.g., David Musteric -&gt; dmusteric@). Tested against the 47 franchises whose emails ARE published: the pattern matched 38 (~81%). Misses were mostly couples where the address uses the other spouse (e.g., Lori &amp; Tracy Allen -&gt; tallen@), so co-owned franchises also get an Alternate Guess. Verify before relying on these (e.g., an email verification service) - some will bounce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>All 789 about/contact/in-the-news subpages of every location were also crawled; none published a franchise email (only corporate addresses such as pr@).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
           <t>Excluded</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>A "Placeholder Site 2" test entry under Alabama, and one duplicate Trenton, NJ listing.</t>
         </is>

</xml_diff>